<commit_message>
auto: feat: 编辑工具v2升级 + kill_process杀进程树修复
</commit_message>
<xml_diff>
--- a/internal/agent/test.xlsx
+++ b/internal/agent/test.xlsx
@@ -10,6 +10,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="4">
   <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>A</t>
   </si>
   <si>
@@ -17,9 +20,6 @@
   </si>
   <si>
     <t>B</t>
-  </si>
-  <si>
-    <t>2</t>
   </si>
 </sst>
 </file>
@@ -45,18 +45,18 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test: add 4 new unit tests for parallel reject error hooks
</commit_message>
<xml_diff>
--- a/internal/agent/test.xlsx
+++ b/internal/agent/test.xlsx
@@ -10,9 +10,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="4">
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -20,6 +17,9 @@
   </si>
   <si>
     <t>B</t>
+  </si>
+  <si>
+    <t>2</t>
   </si>
 </sst>
 </file>
@@ -45,18 +45,18 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: fix: debug_start 修复 — 移除 dlv dap 命令行 --program 参数 +
</commit_message>
<xml_diff>
--- a/internal/agent/test.xlsx
+++ b/internal/agent/test.xlsx
@@ -10,6 +10,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="4">
   <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>A</t>
   </si>
   <si>
@@ -17,9 +20,6 @@
   </si>
   <si>
     <t>B</t>
-  </si>
-  <si>
-    <t>2</t>
   </si>
 </sst>
 </file>
@@ -45,18 +45,18 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: fix: run_command 改用后台启动+轮询 — 不阻塞 agent
</commit_message>
<xml_diff>
--- a/internal/agent/test.xlsx
+++ b/internal/agent/test.xlsx
@@ -10,16 +10,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="4">
   <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
     <t>A</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>B</t>
   </si>
 </sst>
 </file>
@@ -45,18 +45,18 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>